<commit_message>
Rilis v6.8.2 — unit Description, hapus Merk/Tipe, bulk delete unit customer.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/TMS_Template_Customer_Units.xlsx
+++ b/templates/TMS_Template_Customer_Units.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Customer Units" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,7 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Unit Name</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -449,25 +449,15 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Merk</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>